<commit_message>
Week 5: Complete Login
</commit_message>
<xml_diff>
--- a/Data/PaymentWallet.xlsx
+++ b/Data/PaymentWallet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\PaymentWallet\PaymentWallet\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{320BFAF5-B5DF-49EC-BB94-CE3922C8413F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3346AA81-BA9B-4E40-8ED8-B1906F27983F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -595,7 +595,7 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C3" t="s">
@@ -647,6 +647,7 @@
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B4" r:id="rId2" xr:uid="{F77BA3D6-92CF-458C-91C8-8C0FF997A789}"/>
+    <hyperlink ref="B3" r:id="rId3" xr:uid="{FF28393D-8E4D-4C6C-A248-BC7ED122F74C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Week 6: BCrypting Password Hashing, FundingMethod, AddMoney, Transactions Tracking
</commit_message>
<xml_diff>
--- a/Data/PaymentWallet.xlsx
+++ b/Data/PaymentWallet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\PaymentWallet\PaymentWallet\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3346AA81-BA9B-4E40-8ED8-B1906F27983F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62E588FA-9B0C-47F4-AF63-2838FA538CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="47">
   <si>
     <t>UserID</t>
   </si>
@@ -69,64 +69,55 @@
     <t>CreatedDate</t>
   </si>
   <si>
-    <t>john@gmail.com</t>
-  </si>
-  <si>
-    <t>User1@123</t>
+    <t>Admin1@paywallet.com</t>
+  </si>
+  <si>
+    <t>$2a$11$w5JT75zqZ2zXOTgj8fC37uSaZxLBOdqyj7VTH1pFtYQP1zpnvU4mC</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>Admin User2</t>
+  </si>
+  <si>
+    <t>9999900000</t>
+  </si>
+  <si>
+    <t>21-09-2026</t>
+  </si>
+  <si>
+    <t>user@paywallet.com</t>
+  </si>
+  <si>
+    <t>$2a$11$JMSsv6LPYKz3EJy3mzAWYOC2zianWwZBcf3GEQtnEuubzF.AaEk.e</t>
   </si>
   <si>
     <t>User</t>
   </si>
   <si>
-    <t>TRUE</t>
-  </si>
-  <si>
-    <t>John Doe</t>
-  </si>
-  <si>
-    <t>9999999999</t>
+    <t>User2</t>
+  </si>
+  <si>
+    <t>9999933333</t>
+  </si>
+  <si>
+    <t>AccountID</t>
+  </si>
+  <si>
+    <t>AccountName</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>My Main Account</t>
   </si>
   <si>
     <t>16-09-2026</t>
-  </si>
-  <si>
-    <t>Admin@123</t>
-  </si>
-  <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>Admin User</t>
-  </si>
-  <si>
-    <t>Admin1@gmail.com</t>
-  </si>
-  <si>
-    <t>Admin1@paywallet.com</t>
-  </si>
-  <si>
-    <t>#Admin@123</t>
-  </si>
-  <si>
-    <t>Admin User2</t>
-  </si>
-  <si>
-    <t>9999900000</t>
-  </si>
-  <si>
-    <t>17-09-2026</t>
-  </si>
-  <si>
-    <t>AccountID</t>
-  </si>
-  <si>
-    <t>AccountName</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>My Main Account</t>
   </si>
   <si>
     <t>Active</t>
@@ -528,7 +519,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.81640625" customWidth="1"/>
@@ -566,89 +557,67 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2">
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B5" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C5" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D5" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E5" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F5" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G5" t="s">
         <v>13</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="G6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="B4" r:id="rId2" xr:uid="{F77BA3D6-92CF-458C-91C8-8C0FF997A789}"/>
-    <hyperlink ref="B3" r:id="rId3" xr:uid="{FF28393D-8E4D-4C6C-A248-BC7ED122F74C}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -665,19 +634,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -688,13 +657,13 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -714,25 +683,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -752,28 +721,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -793,16 +762,16 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -832,31 +801,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -874,22 +843,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -907,22 +876,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>36</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week 6: Final Update
</commit_message>
<xml_diff>
--- a/Data/PaymentWallet.xlsx
+++ b/Data/PaymentWallet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\PaymentWallet\PaymentWallet\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62E588FA-9B0C-47F4-AF63-2838FA538CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC959694-7191-487F-B759-96114DB508BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="Refunds" sheetId="7" r:id="rId7"/>
     <sheet name="Notifications" sheetId="8" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" fullPrecision="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>UserID</t>
   </si>
@@ -105,6 +105,36 @@
     <t>9999933333</t>
   </si>
   <si>
+    <t>smarathe232@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$11$Ig7mPSom2TT3q0smVOhF5uNpbiUyDh8gqJBkORkLdus/4WWYZ79RO</t>
+  </si>
+  <si>
+    <t>Shubham Marathe</t>
+  </si>
+  <si>
+    <t>9898989898</t>
+  </si>
+  <si>
+    <t>23-09-2026</t>
+  </si>
+  <si>
+    <t>sharvilj1997@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$11$Cp8azmNQMtn8WuB/vDxTTuEaHU8t3sBHwtqn1iVLQ6Xv/T8PiRwgG</t>
+  </si>
+  <si>
+    <t>Sharvil Jadhav</t>
+  </si>
+  <si>
+    <t>7767574737</t>
+  </si>
+  <si>
+    <t>24-09-2026</t>
+  </si>
+  <si>
     <t>AccountID</t>
   </si>
   <si>
@@ -123,6 +153,15 @@
     <t>Active</t>
   </si>
   <si>
+    <t>My Secondary Account</t>
+  </si>
+  <si>
+    <t>Overseas Account</t>
+  </si>
+  <si>
+    <t>Sharvil Wallet</t>
+  </si>
+  <si>
     <t>WalletID</t>
   </si>
   <si>
@@ -132,6 +171,12 @@
     <t>Currency</t>
   </si>
   <si>
+    <t>INR</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
     <t>TransactionID</t>
   </si>
   <si>
@@ -150,7 +195,52 @@
     <t>FundingMethodID</t>
   </si>
   <si>
+    <t>BalanceBefore</t>
+  </si>
+  <si>
+    <t>BalanceAfter</t>
+  </si>
+  <si>
+    <t>Credit</t>
+  </si>
+  <si>
+    <t>Added money from Card - **** **** **** 3456</t>
+  </si>
+  <si>
+    <t>23-09-2026 23:49</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Added money from Card - **** **** **** 7654</t>
+  </si>
+  <si>
+    <t>24-09-2026 16:38</t>
+  </si>
+  <si>
+    <t>Added money from Card - **** **** **** 3221</t>
+  </si>
+  <si>
+    <t>24-09-2026 16:57</t>
+  </si>
+  <si>
+    <t>24-09-2026 16:59</t>
+  </si>
+  <si>
     <t>MaskedDetails</t>
+  </si>
+  <si>
+    <t>Card</t>
+  </si>
+  <si>
+    <t>**** **** **** 3456</t>
+  </si>
+  <si>
+    <t>**** **** **** 7654</t>
+  </si>
+  <si>
+    <t>**** **** **** 3221</t>
   </si>
   <si>
     <t>PaymentID</t>
@@ -190,7 +280,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -216,7 +307,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
+        <fgColor theme="8" tint="0.3999755851924192"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -232,12 +323,12 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" applyNumberFormat="0" fontId="1" applyFont="1" fillId="0" applyFill="0" borderId="0" applyBorder="0" applyProtection="0" applyAlignment="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" applyFill="1" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" applyFont="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -519,18 +610,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.81640625" customWidth="1"/>
     <col min="2" max="2" width="21.54296875" customWidth="1"/>
     <col min="3" max="3" width="14.36328125" customWidth="1"/>
     <col min="6" max="6" width="12.08984375" customWidth="1"/>
-    <col min="7" max="7" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" bestFit="1" width="10.81640625" customWidth="1"/>
     <col min="8" max="8" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -556,75 +647,131 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2">
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3">
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4">
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
+    <row r="5">
+      <c r="A5" s="0">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="0" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6">
+    <row r="6">
+      <c r="A6" s="0">
         <v>2</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="0" t="s">
         <v>14</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>3</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="H7" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>4</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B5" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D53FE46B-B3DA-4705-AC94-FE70685D3F44}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.26953125" customWidth="1"/>
@@ -632,48 +779,100 @@
     <col min="4" max="4" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>1</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="E2" t="s">
-        <v>25</v>
+      <c r="E3" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>1</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95364483-600B-4196-BD42-B2277A2C52E4}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -681,78 +880,302 @@
     <col min="6" max="6" width="12.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>22</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>2</v>
+      </c>
+      <c r="C2" s="0">
+        <v>1</v>
+      </c>
+      <c r="D2" s="0">
+        <v>1000</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>1</v>
+      </c>
+      <c r="C3" s="0">
+        <v>1</v>
+      </c>
+      <c r="D3" s="0">
+        <v>25</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0">
+        <v>1</v>
+      </c>
+      <c r="D4" s="0">
+        <v>3000</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0">
+        <v>4</v>
+      </c>
+      <c r="D5" s="0">
+        <v>3630</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{684FCF92-7597-465F-B266-1F92F08DABCF}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="5" max="5" width="10.453125" customWidth="1"/>
     <col min="8" max="8" width="16.36328125" customWidth="1"/>
+    <col min="9" max="9" width="12.90625" customWidth="1"/>
+    <col min="10" max="10" width="14.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>34</v>
+        <v>49</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>2</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="0">
+        <v>25</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="H2" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>3</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="0">
+        <v>3000</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="H3" s="0">
+        <v>2</v>
+      </c>
+      <c r="I3" s="0">
+        <v>0</v>
+      </c>
+      <c r="J3" s="0">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>4</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="0">
+        <v>3400</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="H4" s="0">
+        <v>3</v>
+      </c>
+      <c r="I4" s="0">
+        <v>0</v>
+      </c>
+      <c r="J4" s="0">
+        <v>3400</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>4</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="0">
+        <v>230</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="H5" s="0">
+        <v>3</v>
+      </c>
+      <c r="I5" s="0">
+        <v>3400</v>
+      </c>
+      <c r="J5" s="0">
+        <v>3630</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CAAF4AF-C04C-4B6D-A825-38D8950B9DEC}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -760,18 +1183,18 @@
     <col min="6" max="6" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -780,8 +1203,69 @@
         <v>7</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="0">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>1</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>4</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -799,37 +1283,38 @@
     <col min="9" max="9" width="12.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -841,28 +1326,29 @@
     <col min="2" max="2" width="10.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -874,29 +1360,35 @@
     <col min="1" max="1" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
+</file>
+
+<file path=EPPlusLicense.txt>This workbook was created with the EPPlus library, licensed to PaymentWallet under the Polyform Noncommercial license, see https://polyformproject.org/licenses/noncommercial/1.0.0
+For more information about EPPlus, see https://epplussoftware.com/
+
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
SOLID refactor complete, send/receive payments, currency validation, duplicate wallet prevention.
</commit_message>
<xml_diff>
--- a/Data/PaymentWallet.xlsx
+++ b/Data/PaymentWallet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\PaymentWallet\PaymentWallet\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC959694-7191-487F-B759-96114DB508BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224F2BFC-DED7-4992-B73D-1208C62436E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="Refunds" sheetId="7" r:id="rId7"/>
     <sheet name="Notifications" sheetId="8" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="1" fullPrecision="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="108">
   <si>
     <t>UserID</t>
   </si>
@@ -135,6 +135,45 @@
     <t>24-09-2026</t>
   </si>
   <si>
+    <t>skaushik98@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$11$7kJE3yf2ycCuU88QoGXpAedkN/xJkzGt61FTba8JVDL7Tvy.WjWvq</t>
+  </si>
+  <si>
+    <t>Shefali Kaushik</t>
+  </si>
+  <si>
+    <t>1234567890</t>
+  </si>
+  <si>
+    <t>wasimakram99@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$11$68DB8hK1SA0wituzySyLdOk/oxx7Xs3bSdRVYTTWtnKkUzVfn9Xku</t>
+  </si>
+  <si>
+    <t>Wasim Akram</t>
+  </si>
+  <si>
+    <t>9887766554</t>
+  </si>
+  <si>
+    <t>07-10-2026</t>
+  </si>
+  <si>
+    <t>sanjaysingh1985@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$11$kYeBADZ1MlQbXEWTvUIthe8k9VnKNFCHozuyUqD1QkThK8h7VWgW2</t>
+  </si>
+  <si>
+    <t>Sanjay Singh</t>
+  </si>
+  <si>
+    <t>8776655443</t>
+  </si>
+  <si>
     <t>AccountID</t>
   </si>
   <si>
@@ -162,6 +201,15 @@
     <t>Sharvil Wallet</t>
   </si>
   <si>
+    <t>Rohan Account</t>
+  </si>
+  <si>
+    <t>My Account</t>
+  </si>
+  <si>
+    <t>My Savings Account</t>
+  </si>
+  <si>
     <t>WalletID</t>
   </si>
   <si>
@@ -174,7 +222,7 @@
     <t>INR</t>
   </si>
   <si>
-    <t>USD</t>
+    <t>EUR</t>
   </si>
   <si>
     <t>TransactionID</t>
@@ -228,6 +276,27 @@
     <t>24-09-2026 16:59</t>
   </si>
   <si>
+    <t>Added money from UPI - shekaus98@icici</t>
+  </si>
+  <si>
+    <t>24-09-2026 18:50</t>
+  </si>
+  <si>
+    <t>24-09-2026 18:55</t>
+  </si>
+  <si>
+    <t>Debit</t>
+  </si>
+  <si>
+    <t>Payment sent to Wallet #7 - Test payment</t>
+  </si>
+  <si>
+    <t>07-10-2026 22:28</t>
+  </si>
+  <si>
+    <t>Payment received from Wallet #1 - Test payment</t>
+  </si>
+  <si>
     <t>MaskedDetails</t>
   </si>
   <si>
@@ -243,6 +312,18 @@
     <t>**** **** **** 3221</t>
   </si>
   <si>
+    <t>UPI</t>
+  </si>
+  <si>
+    <t>shekaus98@icici</t>
+  </si>
+  <si>
+    <t>BankAccount</t>
+  </si>
+  <si>
+    <t>****7373</t>
+  </si>
+  <si>
     <t>PaymentID</t>
   </si>
   <si>
@@ -259,6 +340,18 @@
   </si>
   <si>
     <t>CaptureDate</t>
+  </si>
+  <si>
+    <t>LOCAL_a80cf55d</t>
+  </si>
+  <si>
+    <t>07-10-2026 21:44</t>
+  </si>
+  <si>
+    <t>Test payment</t>
+  </si>
+  <si>
+    <t>LOCAL_cd2b939d</t>
   </si>
   <si>
     <t>RefundID</t>
@@ -280,8 +373,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -307,7 +399,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.3999755851924192"/>
+        <fgColor theme="8" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -323,12 +415,12 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" applyNumberFormat="0" fontId="1" applyFont="1" fillId="0" applyFill="0" borderId="0" applyBorder="0" applyProtection="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" applyFill="1" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" applyFont="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -610,18 +702,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.81640625" customWidth="1"/>
     <col min="2" max="2" width="21.54296875" customWidth="1"/>
     <col min="3" max="3" width="14.36328125" customWidth="1"/>
     <col min="6" max="6" width="12.08984375" customWidth="1"/>
-    <col min="7" max="7" bestFit="1" width="10.81640625" customWidth="1"/>
+    <col min="7" max="7" width="10.81640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -647,131 +739,208 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C2" s="2"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B4" s="2"/>
     </row>
-    <row r="5">
-      <c r="A5" s="0">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="0" t="s">
+      <c r="H5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="0">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6">
         <v>2</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" t="s">
         <v>19</v>
       </c>
-      <c r="H6" s="0" t="s">
+      <c r="H6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="0">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7">
         <v>3</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="F7" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="G7" t="s">
         <v>23</v>
       </c>
-      <c r="H7" s="0" t="s">
+      <c r="H7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="0">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8">
         <v>4</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="F8" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="0" t="s">
+      <c r="G8" t="s">
         <v>28</v>
       </c>
-      <c r="H8" s="0" t="s">
+      <c r="H8" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" t="s">
+        <v>37</v>
+      </c>
+      <c r="H10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G11" t="s">
+        <v>42</v>
+      </c>
+      <c r="H11" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B5" r:id="rId1"/>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D53FE46B-B3DA-4705-AC94-FE70685D3F44}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.26953125" customWidth="1"/>
@@ -779,100 +948,150 @@
     <col min="4" max="4" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="0">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0">
-        <v>1</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="0">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="0">
-        <v>1</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3" s="0" t="s">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="0" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="0">
+      <c r="E3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="0">
-        <v>1</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="0" t="s">
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" t="s">
         <v>29</v>
       </c>
-      <c r="E4" s="0" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="0">
+      <c r="E4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="0">
+      <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="0" t="s">
-        <v>35</v>
+      <c r="E8" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95364483-600B-4196-BD42-B2277A2C52E4}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -880,130 +1099,221 @@
     <col min="6" max="6" width="12.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="0">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
         <v>2</v>
       </c>
-      <c r="C2" s="0">
-        <v>1</v>
-      </c>
-      <c r="D2" s="0">
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>800</v>
+      </c>
+      <c r="E2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>25</v>
+      </c>
+      <c r="E3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>3100</v>
+      </c>
+      <c r="E4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>3630</v>
+      </c>
+      <c r="E5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
         <v>1000</v>
       </c>
-      <c r="E2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="F2" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" s="0" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="0">
-        <v>2</v>
-      </c>
-      <c r="B3" s="0">
-        <v>1</v>
-      </c>
-      <c r="C3" s="0">
-        <v>1</v>
-      </c>
-      <c r="D3" s="0">
-        <v>25</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="0" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="0">
-        <v>3</v>
-      </c>
-      <c r="B4" s="0">
-        <v>3</v>
-      </c>
-      <c r="C4" s="0">
-        <v>1</v>
-      </c>
-      <c r="D4" s="0">
-        <v>3000</v>
-      </c>
-      <c r="E4" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" s="0" t="s">
+      <c r="E6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="0" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="0">
-        <v>4</v>
-      </c>
-      <c r="B5" s="0">
-        <v>4</v>
-      </c>
-      <c r="C5" s="0">
-        <v>4</v>
-      </c>
-      <c r="D5" s="0">
-        <v>3630</v>
-      </c>
-      <c r="E5" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="F5" s="0" t="s">
+      <c r="G6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="0" t="s">
-        <v>35</v>
+      <c r="G7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8">
+        <v>200</v>
+      </c>
+      <c r="E8" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <v>7</v>
+      </c>
+      <c r="D9">
+        <v>2000</v>
+      </c>
+      <c r="E9" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" t="s">
+        <v>38</v>
+      </c>
+      <c r="G9" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{684FCF92-7597-465F-B266-1F92F08DABCF}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1013,169 +1323,296 @@
     <col min="10" max="10" width="14.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="0">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
         <v>2</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="D2" s="0">
+      <c r="C2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D2">
         <v>25</v>
       </c>
-      <c r="E2" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="F2" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="G2" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="H2" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="0">
+      <c r="E2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G2" t="s">
+        <v>71</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="0">
+      <c r="B3">
         <v>3</v>
       </c>
-      <c r="C3" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="D3" s="0">
+      <c r="C3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3">
         <v>3000</v>
       </c>
-      <c r="E3" s="0" t="s">
-        <v>56</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>57</v>
-      </c>
-      <c r="G3" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="H3" s="0">
+      <c r="E3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" t="s">
+        <v>73</v>
+      </c>
+      <c r="G3" t="s">
+        <v>71</v>
+      </c>
+      <c r="H3">
         <v>2</v>
       </c>
-      <c r="I3" s="0">
+      <c r="I3">
         <v>0</v>
       </c>
-      <c r="J3" s="0">
+      <c r="J3">
         <v>3000</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="0">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="0">
+      <c r="B4">
         <v>4</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" s="0">
+      <c r="C4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4">
         <v>3400</v>
       </c>
-      <c r="E4" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="G4" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="H4" s="0">
+      <c r="E4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4" t="s">
+        <v>71</v>
+      </c>
+      <c r="H4">
         <v>3</v>
       </c>
-      <c r="I4" s="0">
+      <c r="I4">
         <v>0</v>
       </c>
-      <c r="J4" s="0">
+      <c r="J4">
         <v>3400</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="0">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="0">
+      <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" s="0">
+      <c r="C5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5">
         <v>230</v>
       </c>
-      <c r="E5" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="G5" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="H5" s="0">
+      <c r="E5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" t="s">
+        <v>76</v>
+      </c>
+      <c r="G5" t="s">
+        <v>71</v>
+      </c>
+      <c r="H5">
         <v>3</v>
       </c>
-      <c r="I5" s="0">
+      <c r="I5">
         <v>3400</v>
       </c>
-      <c r="J5" s="0">
+      <c r="J5">
         <v>3630</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6">
+        <v>1000</v>
+      </c>
+      <c r="E6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G6" t="s">
+        <v>71</v>
+      </c>
+      <c r="H6">
+        <v>4</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7">
+        <v>100</v>
+      </c>
+      <c r="E7" t="s">
+        <v>77</v>
+      </c>
+      <c r="F7" t="s">
+        <v>79</v>
+      </c>
+      <c r="G7" t="s">
+        <v>71</v>
+      </c>
+      <c r="H7">
+        <v>4</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D8">
+        <v>100</v>
+      </c>
+      <c r="E8" t="s">
+        <v>81</v>
+      </c>
+      <c r="F8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G8" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>900</v>
+      </c>
+      <c r="J8">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>68</v>
+      </c>
+      <c r="D9">
+        <v>100</v>
+      </c>
+      <c r="E9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" t="s">
+        <v>82</v>
+      </c>
+      <c r="G9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>100</v>
+      </c>
+      <c r="J9">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CAAF4AF-C04C-4B6D-A825-38D8950B9DEC}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -1183,18 +1620,18 @@
     <col min="6" max="6" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -1203,75 +1640,114 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="0">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0">
-        <v>1</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>63</v>
-      </c>
-      <c r="E2" s="0" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="0">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="0">
-        <v>1</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="E3" s="0" t="s">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="0">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="0">
+      <c r="B4">
         <v>4</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="E4" s="0" t="s">
+      <c r="C4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E4" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E988F3C1-0CA5-49DB-AE11-528DB6674FB8}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" customWidth="1"/>
@@ -1283,38 +1759,95 @@
     <col min="9" max="9" width="12.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>93</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>67</v>
+        <v>94</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>68</v>
+        <v>95</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>69</v>
+        <v>96</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>70</v>
+        <v>97</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>100</v>
+      </c>
+      <c r="E2" t="s">
         <v>71</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>47</v>
+      <c r="F2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H2" t="s">
+        <v>100</v>
+      </c>
+      <c r="I2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>7</v>
+      </c>
+      <c r="D3">
+        <v>100</v>
+      </c>
+      <c r="E3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G3" t="s">
+        <v>82</v>
+      </c>
+      <c r="H3" t="s">
+        <v>82</v>
+      </c>
+      <c r="I3" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
@@ -1326,29 +1859,28 @@
     <col min="2" max="2" width="10.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>93</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>73</v>
+        <v>104</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
@@ -1360,35 +1892,29 @@
     <col min="1" max="1" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>105</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>75</v>
+        <v>106</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>76</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
-</file>
-
-<file path=EPPlusLicense.txt>This workbook was created with the EPPlus library, licensed to PaymentWallet under the Polyform Noncommercial license, see https://polyformproject.org/licenses/noncommercial/1.0.0
-For more information about EPPlus, see https://epplussoftware.com/
-
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Admin tab complete with users, accounts, wallets, payments, stats, GetAllUsers endpoint added
</commit_message>
<xml_diff>
--- a/Data/PaymentWallet.xlsx
+++ b/Data/PaymentWallet.xlsx
@@ -22,7 +22,7 @@
     <sheet name="Refunds" sheetId="7" r:id="rId7"/>
     <sheet name="Notifications" sheetId="8" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" fullPrecision="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
   <si>
     <t>UserID</t>
   </si>
@@ -297,6 +297,18 @@
     <t>Payment received from Wallet #1 - Test payment</t>
   </si>
   <si>
+    <t>Payment sent to Wallet #5 - Lunch</t>
+  </si>
+  <si>
+    <t>07-10-2026 23:21</t>
+  </si>
+  <si>
+    <t>Payment received from Wallet #3 - Lunch</t>
+  </si>
+  <si>
+    <t>07-10-2026 23:24</t>
+  </si>
+  <si>
     <t>MaskedDetails</t>
   </si>
   <si>
@@ -352,6 +364,12 @@
   </si>
   <si>
     <t>LOCAL_cd2b939d</t>
+  </si>
+  <si>
+    <t>LOCAL_1227d9f2</t>
+  </si>
+  <si>
+    <t>Lunch</t>
   </si>
   <si>
     <t>RefundID</t>
@@ -373,7 +391,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -399,7 +418,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
+        <fgColor theme="8" tint="0.3999755851924192"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -415,12 +434,12 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" applyNumberFormat="0" fontId="1" applyFont="1" fillId="0" applyFill="0" borderId="0" applyBorder="0" applyProtection="0" applyAlignment="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" applyFill="1" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" applyFont="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -709,11 +728,11 @@
     <col min="2" max="2" width="21.54296875" customWidth="1"/>
     <col min="3" max="3" width="14.36328125" customWidth="1"/>
     <col min="6" max="6" width="12.08984375" customWidth="1"/>
-    <col min="7" max="7" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" bestFit="1" width="10.81640625" customWidth="1"/>
     <col min="8" max="8" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -739,202 +758,203 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2">
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3">
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4">
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5">
+    <row r="5">
+      <c r="A5" s="0">
         <v>1</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="0" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6">
+    <row r="6">
+      <c r="A6" s="0">
         <v>2</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="0" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7">
+    <row r="7">
+      <c r="A7" s="0">
         <v>3</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="0" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8">
+    <row r="8">
+      <c r="A8" s="0">
         <v>4</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="0" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9">
+    <row r="9">
+      <c r="A9" s="0">
         <v>5</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="0" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10">
+    <row r="10">
+      <c r="A10" s="0">
         <v>6</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="0" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11">
+    <row r="11">
+      <c r="A11" s="0">
         <v>7</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="0" t="s">
         <v>41</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="0" t="s">
         <v>42</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="0" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="B5" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -948,7 +968,7 @@
     <col min="4" max="4" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>43</v>
       </c>
@@ -965,127 +985,128 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="2">
+      <c r="A2" s="0">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="s">
         <v>46</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="0" t="s">
         <v>47</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3">
+    <row r="3">
+      <c r="A3" s="0">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B3" s="0">
+        <v>1</v>
+      </c>
+      <c r="C3" s="0" t="s">
         <v>49</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4">
+    <row r="4">
+      <c r="A4" s="0">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B4" s="0">
+        <v>1</v>
+      </c>
+      <c r="C4" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5">
+    <row r="5">
+      <c r="A5" s="0">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="0">
         <v>4</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="0" t="s">
         <v>51</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6">
+    <row r="6">
+      <c r="A6" s="0">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B6" s="0">
+        <v>1</v>
+      </c>
+      <c r="C6" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7">
+    <row r="7">
+      <c r="A7" s="0">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="0">
         <v>5</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="0" t="s">
         <v>53</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8">
+    <row r="8">
+      <c r="A8" s="0">
         <v>7</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="0">
         <v>7</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="0" t="s">
         <v>54</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="0" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -1099,7 +1120,7 @@
     <col min="6" max="6" width="12.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>55</v>
       </c>
@@ -1122,198 +1143,199 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
+    <row r="2">
+      <c r="A2" s="0">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
         <v>2</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
+      <c r="C2" s="0">
+        <v>1</v>
+      </c>
+      <c r="D2" s="0">
         <v>800</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3">
+    <row r="3">
+      <c r="A3" s="0">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>25</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="B3" s="0">
+        <v>1</v>
+      </c>
+      <c r="C3" s="0">
+        <v>1</v>
+      </c>
+      <c r="D3" s="0">
+        <v>100</v>
+      </c>
+      <c r="E3" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4">
+    <row r="4">
+      <c r="A4" s="0">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="0">
         <v>3</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>3100</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="C4" s="0">
+        <v>1</v>
+      </c>
+      <c r="D4" s="0">
+        <v>2850</v>
+      </c>
+      <c r="E4" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5">
+    <row r="5">
+      <c r="A5" s="0">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="0">
         <v>4</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="0">
         <v>4</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="0">
         <v>3630</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6">
+    <row r="6">
+      <c r="A6" s="0">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="0">
         <v>6</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="0">
         <v>5</v>
       </c>
-      <c r="D6">
-        <v>1000</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="D6" s="0">
+        <v>1250</v>
+      </c>
+      <c r="E6" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7">
+    <row r="7">
+      <c r="A7" s="0">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="0">
         <v>6</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="0">
         <v>5</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="0">
         <v>0</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8">
+    <row r="8">
+      <c r="A8" s="0">
         <v>7</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="0">
         <v>6</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="0">
         <v>5</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="0">
         <v>200</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="0" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9">
+    <row r="9">
+      <c r="A9" s="0">
         <v>8</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="0">
         <v>7</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="0">
         <v>7</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="0">
         <v>2000</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="0" t="s">
         <v>58</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="0" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{684FCF92-7597-465F-B266-1F92F08DABCF}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1323,7 +1345,7 @@
     <col min="10" max="10" width="14.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>60</v>
       </c>
@@ -1355,258 +1377,355 @@
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
+    <row r="2">
+      <c r="A2" s="0">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="0">
         <v>25</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="0" t="s">
         <v>69</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3">
+      <c r="H2" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="0">
         <v>3</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="0">
         <v>3000</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="0" t="s">
         <v>72</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="0">
         <v>2</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="0">
         <v>0</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="0">
         <v>3000</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4">
+    <row r="4">
+      <c r="A4" s="0">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="0">
         <v>4</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="0">
         <v>3400</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="0">
         <v>3</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="0">
         <v>0</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="0">
         <v>3400</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5">
+    <row r="5">
+      <c r="A5" s="0">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="0">
         <v>4</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="0">
         <v>230</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="0" t="s">
         <v>76</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="0">
         <v>3</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="0">
         <v>3400</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="0">
         <v>3630</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6">
+    <row r="6">
+      <c r="A6" s="0">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="0">
         <v>5</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="0">
         <v>1000</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="0" t="s">
         <v>77</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="0">
         <v>4</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="0">
         <v>0</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="0">
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7">
+    <row r="7">
+      <c r="A7" s="0">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="0">
         <v>7</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="0">
         <v>100</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="0" t="s">
         <v>77</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="0">
         <v>4</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="0">
         <v>0</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="0">
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8">
+    <row r="8">
+      <c r="A8" s="0">
         <v>7</v>
       </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="B8" s="0">
+        <v>1</v>
+      </c>
+      <c r="C8" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="0">
         <v>100</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="0">
         <v>0</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="0">
         <v>900</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="0">
         <v>800</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9">
+    <row r="9">
+      <c r="A9" s="0">
         <v>8</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="0">
         <v>7</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="0">
         <v>100</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="0">
         <v>0</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="0">
         <v>100</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="0">
         <v>200</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0">
+        <v>3</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="0">
+        <v>250</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="H10" s="0">
+        <v>0</v>
+      </c>
+      <c r="I10" s="0">
+        <v>3100</v>
+      </c>
+      <c r="J10" s="0">
+        <v>2850</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0">
+        <v>5</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="0">
+        <v>250</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="F11" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="G11" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="H11" s="0">
+        <v>0</v>
+      </c>
+      <c r="I11" s="0">
+        <v>1000</v>
+      </c>
+      <c r="J11" s="0">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0">
+        <v>2</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" s="0">
+        <v>75</v>
+      </c>
+      <c r="E12" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="G12" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="H12" s="0">
+        <v>1</v>
+      </c>
+      <c r="I12" s="0">
+        <v>25</v>
+      </c>
+      <c r="J12" s="0">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -1620,7 +1739,7 @@
     <col min="6" max="6" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>65</v>
       </c>
@@ -1631,7 +1750,7 @@
         <v>61</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -1640,114 +1759,115 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E2" t="s">
+    <row r="2">
+      <c r="A2" s="0">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="0" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3">
+    <row r="3">
+      <c r="A3" s="0">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>85</v>
-      </c>
-      <c r="D3" t="s">
-        <v>87</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="B3" s="0">
+        <v>1</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="E3" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="0" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4">
+    <row r="4">
+      <c r="A4" s="0">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="0">
         <v>4</v>
       </c>
-      <c r="C4" t="s">
-        <v>85</v>
-      </c>
-      <c r="D4" t="s">
-        <v>88</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="C4" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="E4" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="0" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5">
+    <row r="5">
+      <c r="A5" s="0">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="0">
         <v>5</v>
       </c>
-      <c r="C5" t="s">
-        <v>89</v>
-      </c>
-      <c r="D5" t="s">
-        <v>90</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="C5" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="E5" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="0" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6">
+    <row r="6">
+      <c r="A6" s="0">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="0">
         <v>7</v>
       </c>
-      <c r="C6" t="s">
-        <v>91</v>
-      </c>
-      <c r="D6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="C6" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="0" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E988F3C1-0CA5-49DB-AE11-528DB6674FB8}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" customWidth="1"/>
@@ -1759,15 +1879,15 @@
     <col min="9" max="9" width="12.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>62</v>
@@ -1776,78 +1896,108 @@
         <v>45</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
+    <row r="2">
+      <c r="A2" s="0">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0">
         <v>3</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="0">
         <v>100</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="F2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="F2" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0">
+        <v>1</v>
+      </c>
+      <c r="C3" s="0">
+        <v>7</v>
+      </c>
+      <c r="D3" s="0">
         <v>100</v>
       </c>
-      <c r="H2" t="s">
-        <v>100</v>
-      </c>
-      <c r="I2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>7</v>
-      </c>
-      <c r="D3">
-        <v>100</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="E3" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="F3" t="s">
-        <v>102</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="F3" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="G3" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="I3" t="s">
-        <v>101</v>
+      <c r="I3" s="0" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0">
+        <v>3</v>
+      </c>
+      <c r="C4" s="0">
+        <v>5</v>
+      </c>
+      <c r="D4" s="0">
+        <v>250</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="H4" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="I4" s="0" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -1859,18 +2009,18 @@
     <col min="2" max="2" width="10.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>62</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>45</v>
@@ -1881,6 +2031,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -1892,9 +2043,9 @@
     <col min="1" max="1" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1903,18 +2054,24 @@
         <v>61</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>64</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
+</file>
+
+<file path=EPPlusLicense.txt>This workbook was created with the EPPlus library, licensed to PaymentWallet under the Polyform Noncommercial license, see https://polyformproject.org/licenses/noncommercial/1.0.0
+For more information about EPPlus, see https://epplussoftware.com/
+
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Complete features updated. refund flow, email notification, reconciliation, SOLID Architecture
</commit_message>
<xml_diff>
--- a/Data/PaymentWallet.xlsx
+++ b/Data/PaymentWallet.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{224F2BFC-DED7-4992-B73D-1208C62436E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="154">
   <si>
     <t>UserID</t>
   </si>
@@ -174,6 +174,21 @@
     <t>8776655443</t>
   </si>
   <si>
+    <t>namochai75@gmail.com</t>
+  </si>
+  <si>
+    <t>$2a$11$v5P1ZffrCW1YBiv9gY7M.OxtEjx.BevJIaKRB56QMjcCaup4phQ5.</t>
+  </si>
+  <si>
+    <t>Narendra Modi</t>
+  </si>
+  <si>
+    <t>6554433221</t>
+  </si>
+  <si>
+    <t>09-10-2026</t>
+  </si>
+  <si>
     <t>AccountID</t>
   </si>
   <si>
@@ -210,6 +225,9 @@
     <t>My Savings Account</t>
   </si>
   <si>
+    <t>Narendra Modi Account</t>
+  </si>
+  <si>
     <t>WalletID</t>
   </si>
   <si>
@@ -309,6 +327,75 @@
     <t>07-10-2026 23:24</t>
   </si>
   <si>
+    <t>Payment sent to Wallet #7 - Hyperswitch Test payment</t>
+  </si>
+  <si>
+    <t>08-10-2026 11:31</t>
+  </si>
+  <si>
+    <t>Payment received from Wallet #3 - Hyperswitch Test payment</t>
+  </si>
+  <si>
+    <t>08-10-2026 11:43</t>
+  </si>
+  <si>
+    <t>Payment sent to Wallet #8 - Hyperswitch Test payment</t>
+  </si>
+  <si>
+    <t>08-10-2026 13:36</t>
+  </si>
+  <si>
+    <t>Payment received from Wallet #1 - Hyperswitch Test payment</t>
+  </si>
+  <si>
+    <t>08-10-2026 14:11</t>
+  </si>
+  <si>
+    <t>08-10-2026 14:19</t>
+  </si>
+  <si>
+    <t>08-10-2026 15:21</t>
+  </si>
+  <si>
+    <t>08-10-2026 22:53</t>
+  </si>
+  <si>
+    <t>08-10-2026 23:13</t>
+  </si>
+  <si>
+    <t>Refund received - Test Refund</t>
+  </si>
+  <si>
+    <t>08-10-2026 23:27</t>
+  </si>
+  <si>
+    <t>Refund issued - Test Refund</t>
+  </si>
+  <si>
+    <t>Added money from Card - **** **** **** 6378</t>
+  </si>
+  <si>
+    <t>09-10-2026 01:06</t>
+  </si>
+  <si>
+    <t>Payment sent to Wallet #1 - Lunch</t>
+  </si>
+  <si>
+    <t>09-10-2026 01:08</t>
+  </si>
+  <si>
+    <t>Payment received from Wallet #9 - Lunch</t>
+  </si>
+  <si>
+    <t>Refund approved by Admin</t>
+  </si>
+  <si>
+    <t>09-10-2026 01:09</t>
+  </si>
+  <si>
+    <t>Refund deducted - Admin approved</t>
+  </si>
+  <si>
     <t>MaskedDetails</t>
   </si>
   <si>
@@ -336,6 +423,9 @@
     <t>****7373</t>
   </si>
   <si>
+    <t>**** **** **** 6378</t>
+  </si>
+  <si>
     <t>PaymentID</t>
   </si>
   <si>
@@ -370,6 +460,36 @@
   </si>
   <si>
     <t>Lunch</t>
+  </si>
+  <si>
+    <t>Authorized</t>
+  </si>
+  <si>
+    <t>LOCAL_3b1c4183</t>
+  </si>
+  <si>
+    <t>Hyperswitch Test payment</t>
+  </si>
+  <si>
+    <t>LOCAL_91cb3a78</t>
+  </si>
+  <si>
+    <t>LOCAL_442aa996</t>
+  </si>
+  <si>
+    <t>LOCAL_6fc26581</t>
+  </si>
+  <si>
+    <t>LOCAL_57d19128</t>
+  </si>
+  <si>
+    <t>Refunded</t>
+  </si>
+  <si>
+    <t>pay_8a6Kv3TLPxwQH4evzuE3</t>
+  </si>
+  <si>
+    <t>pay_MvabpG9TG7bpIwblFs3M</t>
   </si>
   <si>
     <t>RefundID</t>
@@ -721,7 +841,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.81640625" customWidth="1"/>
@@ -949,6 +1069,32 @@
         <v>38</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="0">
+        <v>8</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="H12" s="0" t="s">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B5" r:id="rId1"/>
@@ -960,7 +1106,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D53FE46B-B3DA-4705-AC94-FE70685D3F44}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.26953125" customWidth="1"/>
@@ -970,19 +1116,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2">
@@ -993,13 +1139,13 @@
         <v>1</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3">
@@ -1010,13 +1156,13 @@
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D3" s="0" t="s">
         <v>24</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -1027,13 +1173,13 @@
         <v>1</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D4" s="0" t="s">
         <v>29</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5">
@@ -1044,13 +1190,13 @@
         <v>4</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D5" s="0" t="s">
         <v>29</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6">
@@ -1061,13 +1207,13 @@
         <v>1</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D6" s="0" t="s">
         <v>29</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7">
@@ -1078,13 +1224,13 @@
         <v>5</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D7" s="0" t="s">
         <v>29</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8">
@@ -1095,13 +1241,30 @@
         <v>7</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D8" s="0" t="s">
         <v>38</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0">
+        <v>8</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1112,7 +1275,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95364483-600B-4196-BD42-B2277A2C52E4}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1122,25 +1285,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2">
@@ -1154,16 +1317,16 @@
         <v>1</v>
       </c>
       <c r="D2" s="0">
-        <v>800</v>
+        <v>650</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F2" s="0" t="s">
         <v>24</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3">
@@ -1180,13 +1343,13 @@
         <v>100</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F3" s="0" t="s">
         <v>24</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -1200,16 +1363,16 @@
         <v>1</v>
       </c>
       <c r="D4" s="0">
-        <v>2850</v>
+        <v>2650</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F4" s="0" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5">
@@ -1226,13 +1389,13 @@
         <v>3630</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F5" s="0" t="s">
         <v>29</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6">
@@ -1249,13 +1412,13 @@
         <v>1250</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F6" s="0" t="s">
         <v>29</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7">
@@ -1272,13 +1435,13 @@
         <v>0</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F7" s="0" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8">
@@ -1292,16 +1455,16 @@
         <v>5</v>
       </c>
       <c r="D8" s="0">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F8" s="0" t="s">
         <v>29</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9">
@@ -1315,16 +1478,39 @@
         <v>7</v>
       </c>
       <c r="D9" s="0">
-        <v>2000</v>
+        <v>2300</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F9" s="0" t="s">
         <v>38</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>48</v>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0">
+        <v>8</v>
+      </c>
+      <c r="C10" s="0">
+        <v>8</v>
+      </c>
+      <c r="D10" s="0">
+        <v>20000</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" s="0" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1335,7 +1521,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{684FCF92-7597-465F-B266-1F92F08DABCF}">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1347,34 +1533,34 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2">
@@ -1385,19 +1571,19 @@
         <v>2</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D2" s="0">
         <v>25</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H2" s="0">
         <v>1</v>
@@ -1411,19 +1597,19 @@
         <v>3</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D3" s="0">
         <v>3000</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H3" s="0">
         <v>2</v>
@@ -1443,19 +1629,19 @@
         <v>4</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D4" s="0">
         <v>3400</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H4" s="0">
         <v>3</v>
@@ -1475,19 +1661,19 @@
         <v>4</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D5" s="0">
         <v>230</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H5" s="0">
         <v>3</v>
@@ -1507,19 +1693,19 @@
         <v>5</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D6" s="0">
         <v>1000</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H6" s="0">
         <v>4</v>
@@ -1539,19 +1725,19 @@
         <v>7</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D7" s="0">
         <v>100</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H7" s="0">
         <v>4</v>
@@ -1571,19 +1757,19 @@
         <v>1</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="D8" s="0">
         <v>100</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H8" s="0">
         <v>0</v>
@@ -1603,19 +1789,19 @@
         <v>7</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D9" s="0">
         <v>100</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H9" s="0">
         <v>0</v>
@@ -1635,19 +1821,19 @@
         <v>3</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="D10" s="0">
         <v>250</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H10" s="0">
         <v>0</v>
@@ -1667,19 +1853,19 @@
         <v>5</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D11" s="0">
         <v>250</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H11" s="0">
         <v>0</v>
@@ -1699,19 +1885,19 @@
         <v>2</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="D12" s="0">
         <v>75</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H12" s="0">
         <v>1</v>
@@ -1721,6 +1907,678 @@
       </c>
       <c r="J12" s="0">
         <v>100</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0">
+        <v>3</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="D13" s="0">
+        <v>100</v>
+      </c>
+      <c r="E13" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="F13" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="G13" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H13" s="0">
+        <v>0</v>
+      </c>
+      <c r="I13" s="0">
+        <v>2850</v>
+      </c>
+      <c r="J13" s="0">
+        <v>2750</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0">
+        <v>7</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" s="0">
+        <v>100</v>
+      </c>
+      <c r="E14" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F14" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="G14" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H14" s="0">
+        <v>0</v>
+      </c>
+      <c r="I14" s="0">
+        <v>200</v>
+      </c>
+      <c r="J14" s="0">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0">
+        <v>3</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="D15" s="0">
+        <v>100</v>
+      </c>
+      <c r="E15" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="F15" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G15" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H15" s="0">
+        <v>0</v>
+      </c>
+      <c r="I15" s="0">
+        <v>2750</v>
+      </c>
+      <c r="J15" s="0">
+        <v>2650</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0">
+        <v>7</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="0">
+        <v>100</v>
+      </c>
+      <c r="E16" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="F16" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="G16" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H16" s="0">
+        <v>0</v>
+      </c>
+      <c r="I16" s="0">
+        <v>300</v>
+      </c>
+      <c r="J16" s="0">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0">
+        <v>1</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" s="0">
+        <v>150</v>
+      </c>
+      <c r="E17" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F17" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G17" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H17" s="0">
+        <v>0</v>
+      </c>
+      <c r="I17" s="0">
+        <v>800</v>
+      </c>
+      <c r="J17" s="0">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0">
+        <v>8</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="D18" s="0">
+        <v>150</v>
+      </c>
+      <c r="E18" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="F18" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="G18" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H18" s="0">
+        <v>0</v>
+      </c>
+      <c r="I18" s="0">
+        <v>2000</v>
+      </c>
+      <c r="J18" s="0">
+        <v>2150</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0">
+        <v>1</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="D19" s="0">
+        <v>100</v>
+      </c>
+      <c r="E19" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F19" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="G19" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H19" s="0">
+        <v>0</v>
+      </c>
+      <c r="I19" s="0">
+        <v>650</v>
+      </c>
+      <c r="J19" s="0">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0">
+        <v>8</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="D20" s="0">
+        <v>100</v>
+      </c>
+      <c r="E20" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="F20" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="G20" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H20" s="0">
+        <v>0</v>
+      </c>
+      <c r="I20" s="0">
+        <v>2150</v>
+      </c>
+      <c r="J20" s="0">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0">
+        <v>1</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" s="0">
+        <v>50</v>
+      </c>
+      <c r="E21" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F21" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="G21" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H21" s="0">
+        <v>0</v>
+      </c>
+      <c r="I21" s="0">
+        <v>550</v>
+      </c>
+      <c r="J21" s="0">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0">
+        <v>8</v>
+      </c>
+      <c r="C22" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="D22" s="0">
+        <v>50</v>
+      </c>
+      <c r="E22" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="F22" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="G22" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H22" s="0">
+        <v>0</v>
+      </c>
+      <c r="I22" s="0">
+        <v>2250</v>
+      </c>
+      <c r="J22" s="0">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0">
+        <v>1</v>
+      </c>
+      <c r="C23" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="D23" s="0">
+        <v>50</v>
+      </c>
+      <c r="E23" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="F23" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="G23" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H23" s="0">
+        <v>0</v>
+      </c>
+      <c r="I23" s="0">
+        <v>500</v>
+      </c>
+      <c r="J23" s="0">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0">
+        <v>8</v>
+      </c>
+      <c r="C24" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" s="0">
+        <v>50</v>
+      </c>
+      <c r="E24" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="F24" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="G24" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H24" s="0">
+        <v>0</v>
+      </c>
+      <c r="I24" s="0">
+        <v>2300</v>
+      </c>
+      <c r="J24" s="0">
+        <v>2350</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0">
+        <v>1</v>
+      </c>
+      <c r="C25" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="D25" s="0">
+        <v>100</v>
+      </c>
+      <c r="E25" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="F25" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="G25" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H25" s="0">
+        <v>1</v>
+      </c>
+      <c r="I25" s="0">
+        <v>450</v>
+      </c>
+      <c r="J25" s="0">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0">
+        <v>1</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="D26" s="0">
+        <v>50</v>
+      </c>
+      <c r="E26" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="F26" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="G26" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H26" s="0">
+        <v>1</v>
+      </c>
+      <c r="I26" s="0">
+        <v>550</v>
+      </c>
+      <c r="J26" s="0">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0">
+        <v>1</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" s="0">
+        <v>50</v>
+      </c>
+      <c r="E27" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="F27" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="G27" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H27" s="0">
+        <v>0</v>
+      </c>
+      <c r="I27" s="0">
+        <v>600</v>
+      </c>
+      <c r="J27" s="0">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0">
+        <v>8</v>
+      </c>
+      <c r="C28" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="D28" s="0">
+        <v>50</v>
+      </c>
+      <c r="E28" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="F28" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="G28" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H28" s="0">
+        <v>0</v>
+      </c>
+      <c r="I28" s="0">
+        <v>2350</v>
+      </c>
+      <c r="J28" s="0">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0">
+        <v>9</v>
+      </c>
+      <c r="C29" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="D29" s="0">
+        <v>20000</v>
+      </c>
+      <c r="E29" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="F29" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="G29" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H29" s="0">
+        <v>6</v>
+      </c>
+      <c r="I29" s="0">
+        <v>0</v>
+      </c>
+      <c r="J29" s="0">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0">
+        <v>9</v>
+      </c>
+      <c r="C30" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="D30" s="0">
+        <v>1000</v>
+      </c>
+      <c r="E30" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="F30" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="G30" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H30" s="0">
+        <v>0</v>
+      </c>
+      <c r="I30" s="0">
+        <v>20000</v>
+      </c>
+      <c r="J30" s="0">
+        <v>19000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0">
+        <v>1</v>
+      </c>
+      <c r="C31" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="D31" s="0">
+        <v>1000</v>
+      </c>
+      <c r="E31" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="F31" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="G31" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H31" s="0">
+        <v>0</v>
+      </c>
+      <c r="I31" s="0">
+        <v>650</v>
+      </c>
+      <c r="J31" s="0">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0">
+        <v>9</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="D32" s="0">
+        <v>1000</v>
+      </c>
+      <c r="E32" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="F32" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="G32" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H32" s="0">
+        <v>0</v>
+      </c>
+      <c r="I32" s="0">
+        <v>19000</v>
+      </c>
+      <c r="J32" s="0">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0">
+        <v>1</v>
+      </c>
+      <c r="C33" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="D33" s="0">
+        <v>1000</v>
+      </c>
+      <c r="E33" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="F33" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="G33" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="H33" s="0">
+        <v>0</v>
+      </c>
+      <c r="I33" s="0">
+        <v>1650</v>
+      </c>
+      <c r="J33" s="0">
+        <v>650</v>
       </c>
     </row>
   </sheetData>
@@ -1731,7 +2589,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CAAF4AF-C04C-4B6D-A825-38D8950B9DEC}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -1741,16 +2599,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>88</v>
+        <v>117</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -1767,10 +2625,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>90</v>
+        <v>119</v>
       </c>
       <c r="E2" s="0" t="s">
         <v>11</v>
@@ -1787,10 +2645,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>91</v>
+        <v>120</v>
       </c>
       <c r="E3" s="0" t="s">
         <v>11</v>
@@ -1807,10 +2665,10 @@
         <v>4</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>92</v>
+        <v>121</v>
       </c>
       <c r="E4" s="0" t="s">
         <v>11</v>
@@ -1827,10 +2685,10 @@
         <v>5</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>93</v>
+        <v>122</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>94</v>
+        <v>123</v>
       </c>
       <c r="E5" s="0" t="s">
         <v>11</v>
@@ -1847,16 +2705,36 @@
         <v>7</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>95</v>
+        <v>124</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>96</v>
+        <v>125</v>
       </c>
       <c r="E6" s="0" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="0" t="s">
         <v>38</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0">
+        <v>8</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1867,7 +2745,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E988F3C1-0CA5-49DB-AE11-528DB6674FB8}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.7265625" customWidth="1"/>
@@ -1881,31 +2759,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>99</v>
+        <v>129</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2">
@@ -1922,19 +2800,19 @@
         <v>100</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>103</v>
+        <v>133</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>105</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3">
@@ -1951,19 +2829,19 @@
         <v>100</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>105</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4">
@@ -1980,19 +2858,207 @@
         <v>250</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>107</v>
+        <v>137</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>108</v>
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0">
+        <v>3</v>
+      </c>
+      <c r="C5" s="0">
+        <v>7</v>
+      </c>
+      <c r="D5" s="0">
+        <v>100</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>140</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="I5" s="0" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0">
+        <v>3</v>
+      </c>
+      <c r="C6" s="0">
+        <v>7</v>
+      </c>
+      <c r="D6" s="0">
+        <v>100</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="F6" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="G6" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="I6" s="0" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0">
+        <v>1</v>
+      </c>
+      <c r="C7" s="0">
+        <v>8</v>
+      </c>
+      <c r="D7" s="0">
+        <v>150</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="G7" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="I7" s="0" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0">
+        <v>1</v>
+      </c>
+      <c r="C8" s="0">
+        <v>8</v>
+      </c>
+      <c r="D8" s="0">
+        <v>100</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="F8" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="G8" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="I8" s="0" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0">
+        <v>1</v>
+      </c>
+      <c r="C9" s="0">
+        <v>8</v>
+      </c>
+      <c r="D9" s="0">
+        <v>50</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="F9" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="G9" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="I9" s="0" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0">
+        <v>1</v>
+      </c>
+      <c r="C10" s="0">
+        <v>8</v>
+      </c>
+      <c r="D10" s="0">
+        <v>50</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="F10" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="G10" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="H10" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="I10" s="0" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0">
+        <v>9</v>
+      </c>
+      <c r="C11" s="0">
+        <v>1</v>
+      </c>
+      <c r="D11" s="0">
+        <v>1000</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="F11" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="G11" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="H11" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="I11" s="0" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -2011,22 +3077,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -2045,22 +3111,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>111</v>
+        <v>151</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>112</v>
+        <v>152</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>113</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>